<commit_message>
Chore:SAP SPP ShPP content added
</commit_message>
<xml_diff>
--- a/Calculation demo/SMP_Calculation.xlsx
+++ b/Calculation demo/SMP_Calculation.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UK-Payroll\Statutory Leave and Pay\Calculation demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB40E8A-021D-480C-A7F1-0FB2524DF7BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BDFCF7F-C3C5-4C9F-92E7-4F417D063F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{54BACE44-3DFD-4A4B-8686-A0AF3799897D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{54BACE44-3DFD-4A4B-8686-A0AF3799897D}"/>
   </bookViews>
   <sheets>
     <sheet name="SMP" sheetId="1" r:id="rId1"/>
-    <sheet name="Alabaster" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Pay Frequency</t>
   </si>
@@ -504,141 +503,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>752460</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>895695</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>3450</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="2" name="Ink 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0B3F6F9-2DD6-43AE-98BB-98FB9F524799}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="15649560" y="4105080"/>
-            <a:ext cx="360" cy="360"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="5" name="Ink 4">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38AE0CA2-0A2C-AE94-B97D-1D76D9EE0EF9}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="15643440" y="4098960"/>
-              <a:ext cx="12600" cy="12600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1133205</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>113910</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>476340</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>114270</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="3" name="Ink 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{738AE107-4A5B-45C2-8E26-155912E44064}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="16973280" y="2037960"/>
-            <a:ext cx="360" cy="360"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="6" name="Ink 5">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{555D5601-56DD-BB40-9AFB-ED3DA3C65645}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="16967160" y="2031840"/>
-              <a:ext cx="12600" cy="12600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
@@ -683,60 +547,6 @@
         </inkml:channelProperties>
       </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2026-05-04T04:47:42.042"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1 24575,'0'0'-8191</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink3.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-05-04T05:52:12.268"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 0 24575,'0'0'-8191</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink4.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-05-04T05:52:12.269"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.035" units="cm"/>
@@ -1187,7 +997,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="29">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="17"/>
@@ -1203,7 +1013,7 @@
       </c>
       <c r="C10" s="31">
         <f>C9/_xlfn.XLOOKUP(C2,F3:F6,G3:G6)</f>
-        <v>4166.666666666667</v>
+        <v>5000</v>
       </c>
       <c r="D10" s="15"/>
       <c r="E10" s="18"/>
@@ -1217,7 +1027,7 @@
       </c>
       <c r="C11" s="32">
         <f>(C10*_xlfn.XLOOKUP(C2,F3:F6,G3:G6))/52</f>
-        <v>961.53846153846155</v>
+        <v>1153.8461538461538</v>
       </c>
       <c r="D11" s="20"/>
       <c r="E11" s="21"/>
@@ -1231,7 +1041,7 @@
       </c>
       <c r="C12" s="29">
         <f>C11*C6</f>
-        <v>865.38461538461536</v>
+        <v>1038.4615384615386</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="17"/>
@@ -1245,7 +1055,7 @@
       </c>
       <c r="C13" s="31">
         <f>C12*C3</f>
-        <v>5192.3076923076924</v>
+        <v>6230.7692307692314</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="23"/>
@@ -1273,7 +1083,7 @@
       </c>
       <c r="C15" s="10">
         <f>C13+C14</f>
-        <v>11604.867692307693</v>
+        <v>12643.329230769232</v>
       </c>
       <c r="D15" s="25"/>
       <c r="E15" s="26"/>
@@ -1329,273 +1139,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5B5D159-04B7-4C4B-9C13-D17D08005F94}">
-  <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="17.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="12.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="34.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.21875" style="1"/>
-    <col min="11" max="11" width="32.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="17.21875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="36">
-        <v>194.32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="33.6" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="4">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="5">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="4">
-        <v>33</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="6">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="4">
-        <f>C3+C4</f>
-        <v>39</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="5">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="7">
-        <v>0.9</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="5">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C7" s="1"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-    </row>
-    <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="B8" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="29">
-        <v>50000</v>
-      </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="3"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="31">
-        <f>$C$9/_xlfn.XLOOKUP($C$2,$F$3:$F$6,$G$3:$G$6)</f>
-        <v>4166.666666666667</v>
-      </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="19"/>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="32">
-        <f>(C10*_xlfn.XLOOKUP(C2,F3:F6,G3:G6))/52</f>
-        <v>961.53846153846155</v>
-      </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="19"/>
-      <c r="J11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="29">
-        <f>C11*C6</f>
-        <v>865.38461538461536</v>
-      </c>
-      <c r="D12" s="20"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="19"/>
-      <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="31">
-        <f>C12*C3</f>
-        <v>5192.3076923076924</v>
-      </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
-      <c r="J13" s="3"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="33" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="31">
-        <f>IF(C11&gt;C1,C1,C11)*C4</f>
-        <v>6412.5599999999995</v>
-      </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-      <c r="J14" s="3"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="10">
-        <f>C13+C14</f>
-        <v>11604.867692307693</v>
-      </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="24"/>
-      <c r="J15" s="3"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C16" s="1"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="11"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C17" s="1"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="11"/>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="11"/>
-    </row>
-    <row r="19" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C19" s="1"/>
-      <c r="G19" s="11"/>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="E20" s="11"/>
-      <c r="G20" s="11"/>
-    </row>
-    <row r="21" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-    </row>
-    <row r="22" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="E22" s="11"/>
-    </row>
-    <row r="26" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-    </row>
-    <row r="27" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="G27" s="11"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>